<commit_message>
Update UniCafe history exports
</commit_message>
<xml_diff>
--- a/data/unicafe-history.xlsx
+++ b/data/unicafe-history.xlsx
@@ -181,8 +181,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UniCafeHistory" displayName="UniCafeHistory" ref="A5:J91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A5:J91"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UniCafeHistory" displayName="UniCafeHistory" ref="A5:J92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A5:J92"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ردیف ثبت"/>
     <tableColumn id="2" name="تاریخ شمسی"/>
@@ -497,9 +497,9 @@
         <v>شناسه ثبت</v>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="16">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
@@ -508,42 +508,48 @@
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:32</t>
+          <t xml:space="preserve">11:25:59</t>
         </is>
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">شارژ و خروج از انبار</t>
+          <t xml:space="preserve">یادداشت و آمار قهوه</t>
         </is>
       </c>
       <c r="E6" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">62</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F6" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">پرو شیر</t>
-        </is>
-      </c>
-      <c r="G6" s="22">
-        <v>4</v>
-      </c>
-      <c r="H6" s="22">
-        <v>0</v>
-      </c>
-      <c r="I6" s="20">
-        <v>4</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">وجین رو یکم ردیفشو خالی کردم به نظر بیاد دوتا فروش رفته خیلی وقته ثابته</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">371938f24f</t>
+          <t xml:space="preserve">2688d62325</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="18">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
@@ -552,7 +558,7 @@
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:29</t>
+          <t xml:space="preserve">09:18:32</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -562,12 +568,12 @@
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">67</t>
+          <t xml:space="preserve">62</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">لایف با قند</t>
+          <t xml:space="preserve">پرو شیر</t>
         </is>
       </c>
       <c r="G7" s="23">
@@ -581,13 +587,13 @@
       </c>
       <c r="J7" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">42a5348cd6</t>
+          <t xml:space="preserve">371938f24f</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="16">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
@@ -596,7 +602,7 @@
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:27</t>
+          <t xml:space="preserve">09:18:29</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
@@ -606,12 +612,12 @@
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">52</t>
+          <t xml:space="preserve">67</t>
         </is>
       </c>
       <c r="F8" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">تیتو مزمز</t>
+          <t xml:space="preserve">لایف با قند</t>
         </is>
       </c>
       <c r="G8" s="22">
@@ -625,13 +631,13 @@
       </c>
       <c r="J8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">326a06b821</t>
+          <t xml:space="preserve">42a5348cd6</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="18">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
@@ -640,7 +646,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:24</t>
+          <t xml:space="preserve">09:18:27</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -650,32 +656,32 @@
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">51</t>
+          <t xml:space="preserve">52</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کیک میک شیفون</t>
+          <t xml:space="preserve">تیتو مزمز</t>
         </is>
       </c>
       <c r="G9" s="23">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H9" s="23">
         <v>0</v>
       </c>
       <c r="I9" s="21">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ad336a97ef</t>
+          <t xml:space="preserve">326a06b821</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="16">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
@@ -684,7 +690,7 @@
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:22</t>
+          <t xml:space="preserve">09:18:24</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
@@ -694,32 +700,32 @@
       </c>
       <c r="E10" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">48</t>
+          <t xml:space="preserve">51</t>
         </is>
       </c>
       <c r="F10" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">پتی بور</t>
+          <t xml:space="preserve">کیک میک شیفون</t>
         </is>
       </c>
       <c r="G10" s="22">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H10" s="22">
         <v>0</v>
       </c>
       <c r="I10" s="20">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J10" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">a805c9c231</t>
+          <t xml:space="preserve">ad336a97ef</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="18">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
@@ -728,7 +734,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:20</t>
+          <t xml:space="preserve">09:18:22</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -738,32 +744,32 @@
       </c>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">41</t>
+          <t xml:space="preserve">48</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">اب معدنی</t>
+          <t xml:space="preserve">پتی بور</t>
         </is>
       </c>
       <c r="G11" s="23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H11" s="23">
         <v>0</v>
       </c>
       <c r="I11" s="21">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J11" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">a8ff3d619f</t>
+          <t xml:space="preserve">a805c9c231</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="16">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
@@ -772,7 +778,7 @@
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:18</t>
+          <t xml:space="preserve">09:18:20</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
@@ -782,32 +788,32 @@
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">36</t>
+          <t xml:space="preserve">41</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">آجیل</t>
+          <t xml:space="preserve">اب معدنی</t>
         </is>
       </c>
       <c r="G12" s="22">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H12" s="22">
         <v>0</v>
       </c>
       <c r="I12" s="20">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J12" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">11722c1ea0</t>
+          <t xml:space="preserve">a8ff3d619f</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="18">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
@@ -816,7 +822,7 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:16</t>
+          <t xml:space="preserve">09:18:18</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -826,32 +832,32 @@
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">35</t>
+          <t xml:space="preserve">36</t>
         </is>
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کلوجه کاکائویی</t>
+          <t xml:space="preserve">آجیل</t>
         </is>
       </c>
       <c r="G13" s="23">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H13" s="23">
         <v>0</v>
       </c>
       <c r="I13" s="21">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J13" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">5891938adf</t>
+          <t xml:space="preserve">11722c1ea0</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="16">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
@@ -860,7 +866,7 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:14</t>
+          <t xml:space="preserve">09:18:16</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
@@ -870,32 +876,32 @@
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">33</t>
+          <t xml:space="preserve">35</t>
         </is>
       </c>
       <c r="F14" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">پاستیل</t>
+          <t xml:space="preserve">کلوجه کاکائویی</t>
         </is>
       </c>
       <c r="G14" s="22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" s="22">
         <v>0</v>
       </c>
       <c r="I14" s="20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">eaaf8a4c01</t>
+          <t xml:space="preserve">5891938adf</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="18">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
@@ -904,7 +910,7 @@
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:12</t>
+          <t xml:space="preserve">09:18:14</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -914,32 +920,32 @@
       </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">32</t>
+          <t xml:space="preserve">33</t>
         </is>
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کوکی</t>
+          <t xml:space="preserve">پاستیل</t>
         </is>
       </c>
       <c r="G15" s="23">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H15" s="23">
         <v>0</v>
       </c>
       <c r="I15" s="21">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">bf94ca7aef</t>
+          <t xml:space="preserve">eaaf8a4c01</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="16">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
@@ -948,7 +954,7 @@
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:11</t>
+          <t xml:space="preserve">09:18:12</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
@@ -958,32 +964,32 @@
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">32</t>
         </is>
       </c>
       <c r="F16" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">کلوچه نادری نارگیلی</t>
+          <t xml:space="preserve">کوکی</t>
         </is>
       </c>
       <c r="G16" s="22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H16" s="22">
         <v>0</v>
       </c>
       <c r="I16" s="20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">c72c97e061</t>
+          <t xml:space="preserve">bf94ca7aef</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="18">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
@@ -992,7 +998,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:09</t>
+          <t xml:space="preserve">09:18:11</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1002,32 +1008,32 @@
       </c>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t xml:space="preserve">26</t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">همپا ادامسی</t>
+          <t xml:space="preserve">کلوچه نادری نارگیلی</t>
         </is>
       </c>
       <c r="G17" s="23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H17" s="23">
         <v>0</v>
       </c>
       <c r="I17" s="21">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">39ac61bdf4</t>
+          <t xml:space="preserve">c72c97e061</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
@@ -1036,7 +1042,7 @@
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:08</t>
+          <t xml:space="preserve">09:18:09</t>
         </is>
       </c>
       <c r="D18" s="17" t="inlineStr">
@@ -1046,32 +1052,32 @@
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">37</t>
+          <t xml:space="preserve">25</t>
         </is>
       </c>
       <c r="F18" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">بادوم زمینی سرکه</t>
+          <t xml:space="preserve">همپا ادامسی</t>
         </is>
       </c>
       <c r="G18" s="22">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H18" s="22">
         <v>0</v>
       </c>
       <c r="I18" s="20">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">42fdd74805</t>
+          <t xml:space="preserve">39ac61bdf4</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
@@ -1080,7 +1086,7 @@
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:06</t>
+          <t xml:space="preserve">09:18:08</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1090,32 +1096,32 @@
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">27</t>
+          <t xml:space="preserve">37</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کلوچه نادری گردویی</t>
+          <t xml:space="preserve">بادوم زمینی سرکه</t>
         </is>
       </c>
       <c r="G19" s="23">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H19" s="23">
         <v>0</v>
       </c>
       <c r="I19" s="21">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">84e74cfe9c</t>
+          <t xml:space="preserve">42fdd74805</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
@@ -1124,7 +1130,7 @@
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:04</t>
+          <t xml:space="preserve">09:18:06</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
@@ -1134,32 +1140,32 @@
       </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">24</t>
+          <t xml:space="preserve">27</t>
         </is>
       </c>
       <c r="F20" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">همپا دراز</t>
+          <t xml:space="preserve">کلوچه نادری گردویی</t>
         </is>
       </c>
       <c r="G20" s="22">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H20" s="22">
         <v>0</v>
       </c>
       <c r="I20" s="20">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">723667cd28</t>
+          <t xml:space="preserve">84e74cfe9c</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
@@ -1168,7 +1174,7 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:18:01</t>
+          <t xml:space="preserve">09:18:04</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -1178,32 +1184,32 @@
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ مرغ</t>
+          <t xml:space="preserve">همپا دراز</t>
         </is>
       </c>
       <c r="G21" s="23">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H21" s="23">
         <v>0</v>
       </c>
       <c r="I21" s="21">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J21" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">8cbfef9090</t>
+          <t xml:space="preserve">723667cd28</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
@@ -1212,7 +1218,7 @@
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:17:58</t>
+          <t xml:space="preserve">09:18:01</t>
         </is>
       </c>
       <c r="D22" s="17" t="inlineStr">
@@ -1222,32 +1228,32 @@
       </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">13</t>
+          <t xml:space="preserve">15</t>
         </is>
       </c>
       <c r="F22" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ انار گردو</t>
+          <t xml:space="preserve">ساندویچ مرغ</t>
         </is>
       </c>
       <c r="G22" s="22">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H22" s="22">
         <v>0</v>
       </c>
       <c r="I22" s="20">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">86145ae381</t>
+          <t xml:space="preserve">8cbfef9090</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
@@ -1256,7 +1262,7 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">09:17:53</t>
+          <t xml:space="preserve">09:17:58</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -1266,46 +1272,46 @@
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">13</t>
         </is>
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">تیتاپ نادری</t>
+          <t xml:space="preserve">ساندویچ انار گردو</t>
         </is>
       </c>
       <c r="G23" s="23">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H23" s="23">
         <v>0</v>
       </c>
       <c r="I23" s="21">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J23" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a5cbafc23</t>
+          <t xml:space="preserve">86145ae381</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1405/07/24</t>
+          <t xml:space="preserve">1405/07/25</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">12:39:32</t>
+          <t xml:space="preserve">09:17:53</t>
         </is>
       </c>
       <c r="D24" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">شارژ و خروج از انبار</t>
         </is>
       </c>
       <c r="E24" s="17" t="inlineStr">
@@ -1319,19 +1325,17 @@
         </is>
       </c>
       <c r="G24" s="22">
+        <v>5</v>
+      </c>
+      <c r="H24" s="22">
         <v>0</v>
       </c>
-      <c r="H24" s="22">
+      <c r="I24" s="20">
         <v>5</v>
       </c>
-      <c r="I24" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">9422c9aa7d</t>
+          <t xml:space="preserve">7a5cbafc23</t>
         </is>
       </c>
     </row>
@@ -1356,19 +1360,19 @@
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">13</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ انار گردو</t>
+          <t xml:space="preserve">تیتاپ نادری</t>
         </is>
       </c>
       <c r="G25" s="23">
         <v>0</v>
       </c>
       <c r="H25" s="23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I25" s="21" t="inlineStr">
         <is>
@@ -1397,7 +1401,7 @@
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E26" s="17" t="inlineStr">
@@ -1410,15 +1414,11 @@
           <t xml:space="preserve">ساندویچ انار گردو</t>
         </is>
       </c>
-      <c r="G26" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ساندویچ</t>
-        </is>
-      </c>
-      <c r="H26" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ساندویچ انار گردو</t>
-        </is>
+      <c r="G26" s="22">
+        <v>0</v>
+      </c>
+      <c r="H26" s="22">
+        <v>3</v>
       </c>
       <c r="I26" s="20" t="inlineStr">
         <is>
@@ -1447,24 +1447,28 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">13</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ مرغ</t>
-        </is>
-      </c>
-      <c r="G27" s="23">
-        <v>0</v>
-      </c>
-      <c r="H27" s="23">
-        <v>6</v>
+          <t xml:space="preserve">ساندویچ انار گردو</t>
+        </is>
+      </c>
+      <c r="G27" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ساندویچ</t>
+        </is>
+      </c>
+      <c r="H27" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ساندویچ انار گردو</t>
+        </is>
       </c>
       <c r="I27" s="21" t="inlineStr">
         <is>
@@ -1493,7 +1497,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -1506,15 +1510,11 @@
           <t xml:space="preserve">ساندویچ مرغ</t>
         </is>
       </c>
-      <c r="G28" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ساندویچ</t>
-        </is>
-      </c>
-      <c r="H28" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ساندویچ مرغ</t>
-        </is>
+      <c r="G28" s="22">
+        <v>0</v>
+      </c>
+      <c r="H28" s="22">
+        <v>6</v>
       </c>
       <c r="I28" s="20" t="inlineStr">
         <is>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
+          <t xml:space="preserve">15</t>
         </is>
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ بندری</t>
+          <t xml:space="preserve">ساندویچ مرغ</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H29" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ بندری</t>
+          <t xml:space="preserve">ساندویچ مرغ</t>
         </is>
       </c>
       <c r="I29" s="21" t="inlineStr">
@@ -1598,22 +1598,22 @@
       </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">21</t>
+          <t xml:space="preserve">17</t>
         </is>
       </c>
       <c r="F30" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">بایودنت نعناع</t>
+          <t xml:space="preserve">ساندویچ بندری</t>
         </is>
       </c>
       <c r="G30" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ساندویچ</t>
         </is>
       </c>
       <c r="H30" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">بایودنت نعناع</t>
+          <t xml:space="preserve">ساندویچ بندری</t>
         </is>
       </c>
       <c r="I30" s="20" t="inlineStr">
@@ -1648,12 +1648,12 @@
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">22</t>
+          <t xml:space="preserve">21</t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">نات بار زرد</t>
+          <t xml:space="preserve">بایودنت نعناع</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="H31" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">نات بار زرد</t>
+          <t xml:space="preserve">بایودنت نعناع</t>
         </is>
       </c>
       <c r="I31" s="21" t="inlineStr">
@@ -1698,12 +1698,12 @@
       </c>
       <c r="E32" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">23</t>
+          <t xml:space="preserve">22</t>
         </is>
       </c>
       <c r="F32" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">بایودنت توتی فروتی</t>
+          <t xml:space="preserve">نات بار زرد</t>
         </is>
       </c>
       <c r="G32" s="22" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="H32" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">بایودنت توتی فروتی</t>
+          <t xml:space="preserve">نات بار زرد</t>
         </is>
       </c>
       <c r="I32" s="20" t="inlineStr">
@@ -1743,24 +1743,28 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">24</t>
+          <t xml:space="preserve">23</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">همپا دراز</t>
-        </is>
-      </c>
-      <c r="G33" s="23">
-        <v>0</v>
-      </c>
-      <c r="H33" s="23">
-        <v>3</v>
+          <t xml:space="preserve">بایودنت توتی فروتی</t>
+        </is>
+      </c>
+      <c r="G33" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H33" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">بایودنت توتی فروتی</t>
+        </is>
       </c>
       <c r="I33" s="21" t="inlineStr">
         <is>
@@ -1789,7 +1793,7 @@
       </c>
       <c r="D34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E34" s="17" t="inlineStr">
@@ -1802,15 +1806,11 @@
           <t xml:space="preserve">همپا دراز</t>
         </is>
       </c>
-      <c r="G34" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H34" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">همپا دراز</t>
-        </is>
+      <c r="G34" s="22">
+        <v>0</v>
+      </c>
+      <c r="H34" s="22">
+        <v>3</v>
       </c>
       <c r="I34" s="20" t="inlineStr">
         <is>
@@ -1839,24 +1839,28 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">همپا ادامسی</t>
-        </is>
-      </c>
-      <c r="G35" s="23">
-        <v>0</v>
-      </c>
-      <c r="H35" s="23">
-        <v>3</v>
+          <t xml:space="preserve">همپا دراز</t>
+        </is>
+      </c>
+      <c r="G35" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H35" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">همپا دراز</t>
+        </is>
       </c>
       <c r="I35" s="21" t="inlineStr">
         <is>
@@ -1885,7 +1889,7 @@
       </c>
       <c r="D36" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E36" s="17" t="inlineStr">
@@ -1898,15 +1902,11 @@
           <t xml:space="preserve">همپا ادامسی</t>
         </is>
       </c>
-      <c r="G36" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H36" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">همپا ادامسی</t>
-        </is>
+      <c r="G36" s="22">
+        <v>0</v>
+      </c>
+      <c r="H36" s="22">
+        <v>3</v>
       </c>
       <c r="I36" s="20" t="inlineStr">
         <is>
@@ -1935,24 +1935,28 @@
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">25</t>
         </is>
       </c>
       <c r="F37" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کلوچه نادری نارگیلی</t>
-        </is>
-      </c>
-      <c r="G37" s="23">
-        <v>0</v>
-      </c>
-      <c r="H37" s="23">
-        <v>5</v>
+          <t xml:space="preserve">همپا ادامسی</t>
+        </is>
+      </c>
+      <c r="G37" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H37" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">همپا ادامسی</t>
+        </is>
       </c>
       <c r="I37" s="21" t="inlineStr">
         <is>
@@ -1981,7 +1985,7 @@
       </c>
       <c r="D38" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E38" s="17" t="inlineStr">
@@ -1994,15 +1998,11 @@
           <t xml:space="preserve">کلوچه نادری نارگیلی</t>
         </is>
       </c>
-      <c r="G38" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H38" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">کلوچه نادری نارگیلی</t>
-        </is>
+      <c r="G38" s="22">
+        <v>0</v>
+      </c>
+      <c r="H38" s="22">
+        <v>5</v>
       </c>
       <c r="I38" s="20" t="inlineStr">
         <is>
@@ -2031,24 +2031,28 @@
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">27</t>
+          <t xml:space="preserve">26</t>
         </is>
       </c>
       <c r="F39" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کلوچه نادری گردویی</t>
-        </is>
-      </c>
-      <c r="G39" s="23">
-        <v>0</v>
-      </c>
-      <c r="H39" s="23">
-        <v>9</v>
+          <t xml:space="preserve">کلوچه نادری نارگیلی</t>
+        </is>
+      </c>
+      <c r="G39" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H39" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">کلوچه نادری نارگیلی</t>
+        </is>
       </c>
       <c r="I39" s="21" t="inlineStr">
         <is>
@@ -2077,7 +2081,7 @@
       </c>
       <c r="D40" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E40" s="17" t="inlineStr">
@@ -2090,15 +2094,11 @@
           <t xml:space="preserve">کلوچه نادری گردویی</t>
         </is>
       </c>
-      <c r="G40" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H40" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">کلوچه نادری گردویی</t>
-        </is>
+      <c r="G40" s="22">
+        <v>0</v>
+      </c>
+      <c r="H40" s="22">
+        <v>9</v>
       </c>
       <c r="I40" s="20" t="inlineStr">
         <is>
@@ -2132,12 +2132,12 @@
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">28</t>
+          <t xml:space="preserve">27</t>
         </is>
       </c>
       <c r="F41" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کروسان</t>
+          <t xml:space="preserve">کلوچه نادری گردویی</t>
         </is>
       </c>
       <c r="G41" s="23" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="H41" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کروسان</t>
+          <t xml:space="preserve">کلوچه نادری گردویی</t>
         </is>
       </c>
       <c r="I41" s="21" t="inlineStr">
@@ -2182,12 +2182,12 @@
       </c>
       <c r="E42" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">31</t>
+          <t xml:space="preserve">28</t>
         </is>
       </c>
       <c r="F42" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">وافل</t>
+          <t xml:space="preserve">کروسان</t>
         </is>
       </c>
       <c r="G42" s="22" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="H42" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">وافل</t>
+          <t xml:space="preserve">کروسان</t>
         </is>
       </c>
       <c r="I42" s="20" t="inlineStr">
@@ -2227,24 +2227,28 @@
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">32</t>
+          <t xml:space="preserve">31</t>
         </is>
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کوکی</t>
-        </is>
-      </c>
-      <c r="G43" s="23">
-        <v>0</v>
-      </c>
-      <c r="H43" s="23">
-        <v>6</v>
+          <t xml:space="preserve">وافل</t>
+        </is>
+      </c>
+      <c r="G43" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H43" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">وافل</t>
+        </is>
       </c>
       <c r="I43" s="21" t="inlineStr">
         <is>
@@ -2273,7 +2277,7 @@
       </c>
       <c r="D44" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E44" s="17" t="inlineStr">
@@ -2286,15 +2290,11 @@
           <t xml:space="preserve">کوکی</t>
         </is>
       </c>
-      <c r="G44" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H44" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">کوکی</t>
-        </is>
+      <c r="G44" s="22">
+        <v>0</v>
+      </c>
+      <c r="H44" s="22">
+        <v>6</v>
       </c>
       <c r="I44" s="20" t="inlineStr">
         <is>
@@ -2323,24 +2323,28 @@
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">33</t>
+          <t xml:space="preserve">32</t>
         </is>
       </c>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">پاستیل</t>
-        </is>
-      </c>
-      <c r="G45" s="23">
-        <v>0</v>
-      </c>
-      <c r="H45" s="23">
-        <v>3</v>
+          <t xml:space="preserve">کوکی</t>
+        </is>
+      </c>
+      <c r="G45" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H45" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">کوکی</t>
+        </is>
       </c>
       <c r="I45" s="21" t="inlineStr">
         <is>
@@ -2369,7 +2373,7 @@
       </c>
       <c r="D46" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E46" s="17" t="inlineStr">
@@ -2382,15 +2386,11 @@
           <t xml:space="preserve">پاستیل</t>
         </is>
       </c>
-      <c r="G46" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H46" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">پاستیل</t>
-        </is>
+      <c r="G46" s="22">
+        <v>0</v>
+      </c>
+      <c r="H46" s="22">
+        <v>3</v>
       </c>
       <c r="I46" s="20" t="inlineStr">
         <is>
@@ -2424,12 +2424,12 @@
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">34</t>
+          <t xml:space="preserve">33</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ویفر نادری کوچیک</t>
+          <t xml:space="preserve">پاستیل</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="H47" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ویفر نادری کوچیک</t>
+          <t xml:space="preserve">پاستیل</t>
         </is>
       </c>
       <c r="I47" s="21" t="inlineStr">
@@ -2469,24 +2469,28 @@
       </c>
       <c r="D48" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E48" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">35</t>
+          <t xml:space="preserve">34</t>
         </is>
       </c>
       <c r="F48" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">کلوجه کاکائویی</t>
-        </is>
-      </c>
-      <c r="G48" s="22">
-        <v>0</v>
-      </c>
-      <c r="H48" s="22">
-        <v>4</v>
+          <t xml:space="preserve">ویفر نادری کوچیک</t>
+        </is>
+      </c>
+      <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ویفر نادری کوچیک</t>
+        </is>
       </c>
       <c r="I48" s="20" t="inlineStr">
         <is>
@@ -2515,7 +2519,7 @@
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
@@ -2528,15 +2532,11 @@
           <t xml:space="preserve">کلوجه کاکائویی</t>
         </is>
       </c>
-      <c r="G49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">کلوجه کاکائویی</t>
-        </is>
+      <c r="G49" s="23">
+        <v>0</v>
+      </c>
+      <c r="H49" s="23">
+        <v>4</v>
       </c>
       <c r="I49" s="21" t="inlineStr">
         <is>
@@ -2565,24 +2565,28 @@
       </c>
       <c r="D50" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E50" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">36</t>
+          <t xml:space="preserve">35</t>
         </is>
       </c>
       <c r="F50" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">آجیل</t>
-        </is>
-      </c>
-      <c r="G50" s="22">
-        <v>0</v>
-      </c>
-      <c r="H50" s="22">
-        <v>6</v>
+          <t xml:space="preserve">کلوجه کاکائویی</t>
+        </is>
+      </c>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">کلوجه کاکائویی</t>
+        </is>
       </c>
       <c r="I50" s="20" t="inlineStr">
         <is>
@@ -2611,7 +2615,7 @@
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -2624,15 +2628,11 @@
           <t xml:space="preserve">آجیل</t>
         </is>
       </c>
-      <c r="G51" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H51" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">آجیل</t>
-        </is>
+      <c r="G51" s="23">
+        <v>0</v>
+      </c>
+      <c r="H51" s="23">
+        <v>6</v>
       </c>
       <c r="I51" s="21" t="inlineStr">
         <is>
@@ -2661,24 +2661,28 @@
       </c>
       <c r="D52" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E52" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">37</t>
+          <t xml:space="preserve">36</t>
         </is>
       </c>
       <c r="F52" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">بادوم زمینی سرکه</t>
-        </is>
-      </c>
-      <c r="G52" s="22">
-        <v>0</v>
-      </c>
-      <c r="H52" s="22">
-        <v>7</v>
+          <t xml:space="preserve">آجیل</t>
+        </is>
+      </c>
+      <c r="G52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">آجیل</t>
+        </is>
       </c>
       <c r="I52" s="20" t="inlineStr">
         <is>
@@ -2707,7 +2711,7 @@
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
@@ -2720,15 +2724,11 @@
           <t xml:space="preserve">بادوم زمینی سرکه</t>
         </is>
       </c>
-      <c r="G53" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H53" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">بادوم زمینی سرکه</t>
-        </is>
+      <c r="G53" s="23">
+        <v>0</v>
+      </c>
+      <c r="H53" s="23">
+        <v>7</v>
       </c>
       <c r="I53" s="21" t="inlineStr">
         <is>
@@ -2762,12 +2762,12 @@
       </c>
       <c r="E54" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">38</t>
+          <t xml:space="preserve">37</t>
         </is>
       </c>
       <c r="F54" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">رول رول</t>
+          <t xml:space="preserve">بادوم زمینی سرکه</t>
         </is>
       </c>
       <c r="G54" s="22" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="H54" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">رول رول</t>
+          <t xml:space="preserve">بادوم زمینی سرکه</t>
         </is>
       </c>
       <c r="I54" s="20" t="inlineStr">
@@ -2807,24 +2807,28 @@
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">41</t>
+          <t xml:space="preserve">38</t>
         </is>
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">اب معدنی</t>
-        </is>
-      </c>
-      <c r="G55" s="23">
-        <v>0</v>
-      </c>
-      <c r="H55" s="23">
-        <v>3</v>
+          <t xml:space="preserve">رول رول</t>
+        </is>
+      </c>
+      <c r="G55" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H55" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">رول رول</t>
+        </is>
       </c>
       <c r="I55" s="21" t="inlineStr">
         <is>
@@ -2853,7 +2857,7 @@
       </c>
       <c r="D56" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E56" s="17" t="inlineStr">
@@ -2866,15 +2870,11 @@
           <t xml:space="preserve">اب معدنی</t>
         </is>
       </c>
-      <c r="G56" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H56" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">اب معدنی</t>
-        </is>
+      <c r="G56" s="22">
+        <v>0</v>
+      </c>
+      <c r="H56" s="22">
+        <v>3</v>
       </c>
       <c r="I56" s="20" t="inlineStr">
         <is>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="E57" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">42</t>
+          <t xml:space="preserve">41</t>
         </is>
       </c>
       <c r="F57" s="23" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="E58" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">43</t>
+          <t xml:space="preserve">42</t>
         </is>
       </c>
       <c r="F58" s="22" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="E59" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">44</t>
+          <t xml:space="preserve">43</t>
         </is>
       </c>
       <c r="F59" s="23" t="inlineStr">
@@ -3058,12 +3058,12 @@
       </c>
       <c r="E60" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">45</t>
+          <t xml:space="preserve">44</t>
         </is>
       </c>
       <c r="F60" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">های بای نادری</t>
+          <t xml:space="preserve">اب معدنی</t>
         </is>
       </c>
       <c r="G60" s="22" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="H60" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">های بای نادری</t>
+          <t xml:space="preserve">اب معدنی</t>
         </is>
       </c>
       <c r="I60" s="20" t="inlineStr">
@@ -3108,12 +3108,12 @@
       </c>
       <c r="E61" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">46</t>
+          <t xml:space="preserve">45</t>
         </is>
       </c>
       <c r="F61" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">توینکلز</t>
+          <t xml:space="preserve">های بای نادری</t>
         </is>
       </c>
       <c r="G61" s="23" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="H61" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">توینکلز</t>
+          <t xml:space="preserve">های بای نادری</t>
         </is>
       </c>
       <c r="I61" s="21" t="inlineStr">
@@ -3158,12 +3158,12 @@
       </c>
       <c r="E62" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">47</t>
+          <t xml:space="preserve">46</t>
         </is>
       </c>
       <c r="F62" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">معینی پور</t>
+          <t xml:space="preserve">توینکلز</t>
         </is>
       </c>
       <c r="G62" s="22" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="H62" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">معینی پور</t>
+          <t xml:space="preserve">توینکلز</t>
         </is>
       </c>
       <c r="I62" s="20" t="inlineStr">
@@ -3203,24 +3203,28 @@
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">48</t>
+          <t xml:space="preserve">47</t>
         </is>
       </c>
       <c r="F63" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">پتی بور</t>
-        </is>
-      </c>
-      <c r="G63" s="23">
-        <v>0</v>
-      </c>
-      <c r="H63" s="23">
-        <v>5</v>
+          <t xml:space="preserve">معینی پور</t>
+        </is>
+      </c>
+      <c r="G63" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H63" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">معینی پور</t>
+        </is>
       </c>
       <c r="I63" s="21" t="inlineStr">
         <is>
@@ -3249,7 +3253,7 @@
       </c>
       <c r="D64" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E64" s="17" t="inlineStr">
@@ -3262,15 +3266,11 @@
           <t xml:space="preserve">پتی بور</t>
         </is>
       </c>
-      <c r="G64" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H64" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">پتی بور</t>
-        </is>
+      <c r="G64" s="22">
+        <v>0</v>
+      </c>
+      <c r="H64" s="22">
+        <v>5</v>
       </c>
       <c r="I64" s="20" t="inlineStr">
         <is>
@@ -3299,24 +3299,28 @@
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">51</t>
+          <t xml:space="preserve">48</t>
         </is>
       </c>
       <c r="F65" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">کیک میک شیفون</t>
-        </is>
-      </c>
-      <c r="G65" s="23">
-        <v>0</v>
-      </c>
-      <c r="H65" s="23">
-        <v>2</v>
+          <t xml:space="preserve">پتی بور</t>
+        </is>
+      </c>
+      <c r="G65" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H65" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پتی بور</t>
+        </is>
       </c>
       <c r="I65" s="21" t="inlineStr">
         <is>
@@ -3345,7 +3349,7 @@
       </c>
       <c r="D66" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E66" s="17" t="inlineStr">
@@ -3358,15 +3362,11 @@
           <t xml:space="preserve">کیک میک شیفون</t>
         </is>
       </c>
-      <c r="G66" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H66" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">کیک میک شیفون</t>
-        </is>
+      <c r="G66" s="22">
+        <v>0</v>
+      </c>
+      <c r="H66" s="22">
+        <v>2</v>
       </c>
       <c r="I66" s="20" t="inlineStr">
         <is>
@@ -3395,24 +3395,28 @@
       </c>
       <c r="D67" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E67" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">52</t>
+          <t xml:space="preserve">51</t>
         </is>
       </c>
       <c r="F67" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">تیتو مزمز</t>
-        </is>
-      </c>
-      <c r="G67" s="23">
-        <v>0</v>
-      </c>
-      <c r="H67" s="23">
-        <v>4</v>
+          <t xml:space="preserve">کیک میک شیفون</t>
+        </is>
+      </c>
+      <c r="G67" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H67" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">کیک میک شیفون</t>
+        </is>
       </c>
       <c r="I67" s="21" t="inlineStr">
         <is>
@@ -3441,7 +3445,7 @@
       </c>
       <c r="D68" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E68" s="17" t="inlineStr">
@@ -3454,15 +3458,11 @@
           <t xml:space="preserve">تیتو مزمز</t>
         </is>
       </c>
-      <c r="G68" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H68" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تیتو مزمز</t>
-        </is>
+      <c r="G68" s="22">
+        <v>0</v>
+      </c>
+      <c r="H68" s="22">
+        <v>4</v>
       </c>
       <c r="I68" s="20" t="inlineStr">
         <is>
@@ -3496,12 +3496,12 @@
       </c>
       <c r="E69" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">53</t>
+          <t xml:space="preserve">52</t>
         </is>
       </c>
       <c r="F69" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">شیر شکلات</t>
+          <t xml:space="preserve">تیتو مزمز</t>
         </is>
       </c>
       <c r="G69" s="23" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="H69" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">شیر شکلات</t>
+          <t xml:space="preserve">تیتو مزمز</t>
         </is>
       </c>
       <c r="I69" s="21" t="inlineStr">
@@ -3546,12 +3546,12 @@
       </c>
       <c r="E70" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">54</t>
+          <t xml:space="preserve">53</t>
         </is>
       </c>
       <c r="F70" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">رول رول با کلاس</t>
+          <t xml:space="preserve">شیر شکلات</t>
         </is>
       </c>
       <c r="G70" s="22" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="H70" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">رول رول با کلاس</t>
+          <t xml:space="preserve">شیر شکلات</t>
         </is>
       </c>
       <c r="I70" s="20" t="inlineStr">
@@ -3596,12 +3596,12 @@
       </c>
       <c r="E71" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">55</t>
+          <t xml:space="preserve">54</t>
         </is>
       </c>
       <c r="F71" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">شیر قهوه</t>
+          <t xml:space="preserve">رول رول با کلاس</t>
         </is>
       </c>
       <c r="G71" s="23" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="H71" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">شیر قهوه</t>
+          <t xml:space="preserve">رول رول با کلاس</t>
         </is>
       </c>
       <c r="I71" s="21" t="inlineStr">
@@ -3646,12 +3646,12 @@
       </c>
       <c r="E72" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">56</t>
+          <t xml:space="preserve">55</t>
         </is>
       </c>
       <c r="F72" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">سان استار انبه</t>
+          <t xml:space="preserve">شیر قهوه</t>
         </is>
       </c>
       <c r="G72" s="22" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="H72" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">سان استار انبه</t>
+          <t xml:space="preserve">شیر قهوه</t>
         </is>
       </c>
       <c r="I72" s="20" t="inlineStr">
@@ -3696,12 +3696,12 @@
       </c>
       <c r="E73" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">57</t>
+          <t xml:space="preserve">56</t>
         </is>
       </c>
       <c r="F73" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">سان استار پرتقال</t>
+          <t xml:space="preserve">سان استار انبه</t>
         </is>
       </c>
       <c r="G73" s="23" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="H73" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">سان استار پرتقال</t>
+          <t xml:space="preserve">سان استار انبه</t>
         </is>
       </c>
       <c r="I73" s="21" t="inlineStr">
@@ -3746,12 +3746,12 @@
       </c>
       <c r="E74" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">58</t>
+          <t xml:space="preserve">57</t>
         </is>
       </c>
       <c r="F74" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">وجین</t>
+          <t xml:space="preserve">سان استار پرتقال</t>
         </is>
       </c>
       <c r="G74" s="22" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="H74" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">وجین</t>
+          <t xml:space="preserve">سان استار پرتقال</t>
         </is>
       </c>
       <c r="I74" s="20" t="inlineStr">
@@ -3796,12 +3796,12 @@
       </c>
       <c r="E75" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">61</t>
+          <t xml:space="preserve">58</t>
         </is>
       </c>
       <c r="F75" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">الوئه ورا</t>
+          <t xml:space="preserve">وجین</t>
         </is>
       </c>
       <c r="G75" s="23" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="H75" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">الوئه ورا</t>
+          <t xml:space="preserve">وجین</t>
         </is>
       </c>
       <c r="I75" s="21" t="inlineStr">
@@ -3841,24 +3841,28 @@
       </c>
       <c r="D76" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E76" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">62</t>
+          <t xml:space="preserve">61</t>
         </is>
       </c>
       <c r="F76" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">پرو شیر</t>
-        </is>
-      </c>
-      <c r="G76" s="22">
-        <v>0</v>
-      </c>
-      <c r="H76" s="22">
-        <v>4</v>
+          <t xml:space="preserve">الوئه ورا</t>
+        </is>
+      </c>
+      <c r="G76" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H76" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الوئه ورا</t>
+        </is>
       </c>
       <c r="I76" s="20" t="inlineStr">
         <is>
@@ -3887,7 +3891,7 @@
       </c>
       <c r="D77" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
@@ -3900,15 +3904,11 @@
           <t xml:space="preserve">پرو شیر</t>
         </is>
       </c>
-      <c r="G77" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H77" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">پرو شیر</t>
-        </is>
+      <c r="G77" s="23">
+        <v>0</v>
+      </c>
+      <c r="H77" s="23">
+        <v>4</v>
       </c>
       <c r="I77" s="21" t="inlineStr">
         <is>
@@ -3942,12 +3942,12 @@
       </c>
       <c r="E78" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">63</t>
+          <t xml:space="preserve">62</t>
         </is>
       </c>
       <c r="F78" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">سن ایچ پت پرتقال</t>
+          <t xml:space="preserve">پرو شیر</t>
         </is>
       </c>
       <c r="G78" s="22" t="inlineStr">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="H78" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">سن ایچ پت پرتقال</t>
+          <t xml:space="preserve">پرو شیر</t>
         </is>
       </c>
       <c r="I78" s="20" t="inlineStr">
@@ -3992,12 +3992,12 @@
       </c>
       <c r="E79" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">64</t>
+          <t xml:space="preserve">63</t>
         </is>
       </c>
       <c r="F79" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ایس مانکی کاکتوس</t>
+          <t xml:space="preserve">سن ایچ پت پرتقال</t>
         </is>
       </c>
       <c r="G79" s="23" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="H79" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ایس مانکی کاکتوس</t>
+          <t xml:space="preserve">سن ایچ پت پرتقال</t>
         </is>
       </c>
       <c r="I79" s="21" t="inlineStr">
@@ -4042,12 +4042,12 @@
       </c>
       <c r="E80" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">65</t>
+          <t xml:space="preserve">64</t>
         </is>
       </c>
       <c r="F80" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">ایس مانکی کیوی</t>
+          <t xml:space="preserve">ایس مانکی کاکتوس</t>
         </is>
       </c>
       <c r="G80" s="22" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="H80" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">ایس مانکی کیوی</t>
+          <t xml:space="preserve">ایس مانکی کاکتوس</t>
         </is>
       </c>
       <c r="I80" s="20" t="inlineStr">
@@ -4092,12 +4092,12 @@
       </c>
       <c r="E81" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">66</t>
+          <t xml:space="preserve">65</t>
         </is>
       </c>
       <c r="F81" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">رانی</t>
+          <t xml:space="preserve">ایس مانکی کیوی</t>
         </is>
       </c>
       <c r="G81" s="23" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="H81" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">رانی</t>
+          <t xml:space="preserve">ایس مانکی کیوی</t>
         </is>
       </c>
       <c r="I81" s="21" t="inlineStr">
@@ -4137,24 +4137,28 @@
       </c>
       <c r="D82" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">تغییر نام محصول</t>
         </is>
       </c>
       <c r="E82" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">67</t>
+          <t xml:space="preserve">66</t>
         </is>
       </c>
       <c r="F82" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">لایف با قند</t>
-        </is>
-      </c>
-      <c r="G82" s="22">
-        <v>0</v>
-      </c>
-      <c r="H82" s="22">
-        <v>4</v>
+          <t xml:space="preserve">رانی</t>
+        </is>
+      </c>
+      <c r="G82" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H82" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">رانی</t>
+        </is>
       </c>
       <c r="I82" s="20" t="inlineStr">
         <is>
@@ -4183,7 +4187,7 @@
       </c>
       <c r="D83" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
@@ -4196,15 +4200,11 @@
           <t xml:space="preserve">لایف با قند</t>
         </is>
       </c>
-      <c r="G83" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H83" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">لایف با قند</t>
-        </is>
+      <c r="G83" s="23">
+        <v>0</v>
+      </c>
+      <c r="H83" s="23">
+        <v>4</v>
       </c>
       <c r="I83" s="21" t="inlineStr">
         <is>
@@ -4238,132 +4238,138 @@
       </c>
       <c r="E84" s="17" t="inlineStr">
         <is>
+          <t xml:space="preserve">67</t>
+        </is>
+      </c>
+      <c r="F84" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">لایف با قند</t>
+        </is>
+      </c>
+      <c r="G84" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H84" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">لایف با قند</t>
+        </is>
+      </c>
+      <c r="I84" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J84" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9422c9aa7d</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="28" customHeight="1">
+      <c r="A85" s="18">
+        <v>3</v>
+      </c>
+      <c r="B85" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1405/07/24</t>
+        </is>
+      </c>
+      <c r="C85" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12:39:32</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تغییر نام محصول</t>
+        </is>
+      </c>
+      <c r="E85" s="19" t="inlineStr">
+        <is>
           <t xml:space="preserve">68</t>
         </is>
       </c>
-      <c r="F84" s="22" t="inlineStr">
+      <c r="F85" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">لایف بدون قند</t>
         </is>
       </c>
-      <c r="G84" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H84" s="22" t="inlineStr">
+      <c r="G85" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H85" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">لایف بدون قند</t>
         </is>
       </c>
-      <c r="I84" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J84" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9422c9aa7d</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="48" customHeight="1">
-      <c r="A85" s="18">
-        <v>3</v>
-      </c>
-      <c r="B85" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1405/07/24</t>
-        </is>
-      </c>
-      <c r="C85" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12:39:32</t>
-        </is>
-      </c>
-      <c r="D85" s="19" t="inlineStr">
+      <c r="I85" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J85" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9422c9aa7d</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="48" customHeight="1">
+      <c r="A86" s="16">
+        <v>3</v>
+      </c>
+      <c r="B86" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1405/07/24</t>
+        </is>
+      </c>
+      <c r="C86" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12:39:32</t>
+        </is>
+      </c>
+      <c r="D86" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">یادداشت و آمار قهوه</t>
         </is>
       </c>
-      <c r="E85" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F85" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G85" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H85" s="23" t="inlineStr">
+      <c r="E86" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F86" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G86" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H86" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">وجین رو یکم ردیفشو خالی کردم به نظر بیاد دوتا فروش رفته خیلی وقته ثابته</t>
         </is>
       </c>
-      <c r="I85" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J85" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9422c9aa7d</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="28" customHeight="1">
-      <c r="A86" s="16">
-        <v>2</v>
-      </c>
-      <c r="B86" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1405/07/23</t>
-        </is>
-      </c>
-      <c r="C86" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23:16:19</t>
-        </is>
-      </c>
-      <c r="D86" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">شارژ و خروج از انبار</t>
-        </is>
-      </c>
-      <c r="E86" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="F86" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تیتاپ نادری</t>
-        </is>
-      </c>
-      <c r="G86" s="22">
-        <v>4</v>
-      </c>
-      <c r="H86" s="22">
-        <v>0</v>
-      </c>
-      <c r="I86" s="20">
-        <v>4</v>
+      <c r="I86" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="J86" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">deac82c691</t>
+          <t xml:space="preserve">9422c9aa7d</t>
         </is>
       </c>
     </row>
     <row r="87" ht="28" customHeight="1">
       <c r="A87" s="18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B87" s="19" t="inlineStr">
         <is>
@@ -4372,12 +4378,12 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">22:41:53</t>
+          <t xml:space="preserve">23:16:19</t>
         </is>
       </c>
       <c r="D87" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ثبت آمار</t>
+          <t xml:space="preserve">شارژ و خروج از انبار</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
@@ -4391,19 +4397,17 @@
         </is>
       </c>
       <c r="G87" s="23">
+        <v>4</v>
+      </c>
+      <c r="H87" s="23">
         <v>0</v>
       </c>
-      <c r="H87" s="23">
+      <c r="I87" s="21">
         <v>4</v>
       </c>
-      <c r="I87" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J87" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">3a58237bc2</t>
+          <t xml:space="preserve">deac82c691</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4427,7 @@
       </c>
       <c r="D88" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">تغییر نام محصول</t>
+          <t xml:space="preserve">ثبت آمار</t>
         </is>
       </c>
       <c r="E88" s="17" t="inlineStr">
@@ -4436,15 +4440,11 @@
           <t xml:space="preserve">تیتاپ نادری</t>
         </is>
       </c>
-      <c r="G88" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H88" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تیتاپ نادری</t>
-        </is>
+      <c r="G88" s="22">
+        <v>0</v>
+      </c>
+      <c r="H88" s="22">
+        <v>4</v>
       </c>
       <c r="I88" s="20" t="inlineStr">
         <is>
@@ -4478,12 +4478,12 @@
       </c>
       <c r="E89" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">13</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="F89" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ</t>
+          <t xml:space="preserve">تیتاپ نادری</t>
         </is>
       </c>
       <c r="G89" s="23" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="H89" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ساندویچ</t>
+          <t xml:space="preserve">تیتاپ نادری</t>
         </is>
       </c>
       <c r="I89" s="21" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="E90" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">13</t>
         </is>
       </c>
       <c r="F90" s="22" t="inlineStr">
@@ -4578,30 +4578,80 @@
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="F91" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ساندویچ</t>
+        </is>
+      </c>
+      <c r="G91" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H91" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ساندویچ</t>
+        </is>
+      </c>
+      <c r="I91" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J91" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3a58237bc2</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="28" customHeight="1">
+      <c r="A92" s="16">
+        <v>1</v>
+      </c>
+      <c r="B92" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1405/07/23</t>
+        </is>
+      </c>
+      <c r="C92" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22:41:53</t>
+        </is>
+      </c>
+      <c r="D92" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تغییر نام محصول</t>
+        </is>
+      </c>
+      <c r="E92" s="17" t="inlineStr">
+        <is>
           <t xml:space="preserve">17</t>
         </is>
       </c>
-      <c r="F91" s="23" t="inlineStr">
+      <c r="F92" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">ساندویچ</t>
         </is>
       </c>
-      <c r="G91" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H91" s="23" t="inlineStr">
+      <c r="G92" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H92" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">ساندویچ</t>
         </is>
       </c>
-      <c r="I91" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J91" s="19" t="inlineStr">
+      <c r="I92" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J92" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">3a58237bc2</t>
         </is>

</xml_diff>